<commit_message>
Enviando demo de como alterar os lançamentos conforme os dados do escritório
</commit_message>
<xml_diff>
--- a/mock_dados_area.xlsx
+++ b/mock_dados_area.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saulo\github\demo-asana_api-comunicapje\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65C2EBB-C7B1-442E-8ADC-05BCDB9B0FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E74489-F00B-49B7-AD4F-8A0084BA2632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4935" yWindow="3195" windowWidth="28800" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
   <si>
     <t>processo</t>
   </si>
@@ -69,27 +69,38 @@
     <t>1045107-93.2025.8.11.0001</t>
   </si>
   <si>
-    <t>ZEZINHO</t>
-  </si>
-  <si>
     <t>area</t>
   </si>
   <si>
     <t>JUIZADO</t>
   </si>
   <si>
-    <t>COMUM-EXEC</t>
-  </si>
-  <si>
-    <t>COMUM-ORD</t>
+    <t>COMUM</t>
+  </si>
+  <si>
+    <t>0000435-03.2025.5.23.0108</t>
+  </si>
+  <si>
+    <t>0000434-18.2025.5.23.0108</t>
+  </si>
+  <si>
+    <t>1021610-32.2025.4.01.3600</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -117,8 +128,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -137,8 +150,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF23BB53-8B47-4F53-8B89-5B93498394B6}" name="Tabela1" displayName="Tabela1" ref="A1:B21" totalsRowShown="0">
-  <autoFilter ref="A1:B21" xr:uid="{BF23BB53-8B47-4F53-8B89-5B93498394B6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF23BB53-8B47-4F53-8B89-5B93498394B6}" name="Tabela1" displayName="Tabela1" ref="A1:B17" totalsRowShown="0">
+  <autoFilter ref="A1:B17" xr:uid="{BF23BB53-8B47-4F53-8B89-5B93498394B6}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E8E84ADD-344B-43FC-8A26-F24B8D6D7C4B}" name="processo"/>
     <tableColumn id="2" xr3:uid="{73B43807-E4EF-403D-84C8-66F4E48EE756}" name="area"/>
@@ -410,185 +423,157 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="B16" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>